<commit_message>
Update 3 okt. 2026 V1
</commit_message>
<xml_diff>
--- a/filer_2/33034474_danske_licens_spil_a_s.xlsx
+++ b/filer_2/33034474_danske_licens_spil_a_s.xlsx
@@ -3787,54 +3787,54 @@
     <row r="74" ht="16" customHeight="1">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>Overskudsgrad (af bruttofortjeneste), %</t>
+          <t>Overskudsgrad, %</t>
         </is>
       </c>
       <c r="B74" s="14">
-        <f>IFERROR(($B$13+$B$15+$B$14)/$B$8*100,"")</f>
+        <f>IFERROR(($B$13+$B$15+$B$14)/$B$4*100,"")</f>
         <v/>
       </c>
       <c r="C74" s="14">
-        <f>IFERROR(($C$13+$C$15+$C$14)/$C$8*100,"")</f>
+        <f>IFERROR(($C$13+$C$15+$C$14)/$C$4*100,"")</f>
         <v/>
       </c>
       <c r="D74" s="14">
-        <f>IFERROR(($D$13+$D$15+$D$14)/$D$8*100,"")</f>
+        <f>IFERROR(($D$13+$D$15+$D$14)/$D$4*100,"")</f>
         <v/>
       </c>
       <c r="E74" s="14">
-        <f>IFERROR(($E$13+$E$15+$E$14)/$E$8*100,"")</f>
+        <f>IFERROR(($E$13+$E$15+$E$14)/$E$4*100,"")</f>
         <v/>
       </c>
       <c r="F74" s="14">
-        <f>IFERROR(($F$13+$F$15+$F$14)/$F$8*100,"")</f>
+        <f>IFERROR(($F$13+$F$15+$F$14)/$F$4*100,"")</f>
         <v/>
       </c>
     </row>
     <row r="75" ht="16" customHeight="1">
       <c r="A75" s="7" t="inlineStr">
         <is>
-          <t>Aktivernes omsætningshastighed (af bruttofortjeneste), gange</t>
+          <t>Aktivernes omsætningshastighed, gange</t>
         </is>
       </c>
       <c r="B75" s="13">
-        <f>IFERROR($B$8/$B$40,"")</f>
+        <f>IFERROR($B$4/$B$40,"")</f>
         <v/>
       </c>
       <c r="C75" s="13">
-        <f>IFERROR($C$8/$C$40,"")</f>
+        <f>IFERROR($C$4/$C$40,"")</f>
         <v/>
       </c>
       <c r="D75" s="13">
-        <f>IFERROR($D$8/$D$40,"")</f>
+        <f>IFERROR($D$4/$D$40,"")</f>
         <v/>
       </c>
       <c r="E75" s="13">
-        <f>IFERROR($E$8/$E$40,"")</f>
+        <f>IFERROR($E$4/$E$40,"")</f>
         <v/>
       </c>
       <c r="F75" s="13">
-        <f>IFERROR($F$8/$F$40,"")</f>
+        <f>IFERROR($F$4/$F$40,"")</f>
         <v/>
       </c>
     </row>
@@ -4246,11 +4246,21 @@
           <t>Nettoomsætning</t>
         </is>
       </c>
-      <c r="B2" s="17" t="n"/>
-      <c r="C2" s="17" t="n"/>
-      <c r="D2" s="17" t="n"/>
-      <c r="E2" s="17" t="n"/>
-      <c r="F2" s="17" t="n"/>
+      <c r="B2" s="17" t="n">
+        <v>1819679</v>
+      </c>
+      <c r="C2" s="17" t="n">
+        <v>1661743</v>
+      </c>
+      <c r="D2" s="17" t="n">
+        <v>1613015</v>
+      </c>
+      <c r="E2" s="17" t="n">
+        <v>1631692</v>
+      </c>
+      <c r="F2" s="17" t="n">
+        <v>1584199</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="16" t="inlineStr">
@@ -4314,11 +4324,21 @@
           <t>Bruttoresultat</t>
         </is>
       </c>
-      <c r="B6" s="17" t="n"/>
-      <c r="C6" s="17" t="n"/>
-      <c r="D6" s="17" t="n"/>
-      <c r="E6" s="17" t="n"/>
-      <c r="F6" s="17" t="n"/>
+      <c r="B6" s="17" t="n">
+        <v>952955</v>
+      </c>
+      <c r="C6" s="17" t="n">
+        <v>896248</v>
+      </c>
+      <c r="D6" s="17" t="n">
+        <v>887375</v>
+      </c>
+      <c r="E6" s="17" t="n">
+        <v>915715</v>
+      </c>
+      <c r="F6" s="17" t="n">
+        <v>896244</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="16" t="inlineStr">
@@ -6137,19 +6157,19 @@
     <row r="34">
       <c r="A34" s="23" t="inlineStr">
         <is>
-          <t>Overskudsgrad (af bruttofortjeneste), %</t>
+          <t>Overskudsgrad, %</t>
         </is>
       </c>
       <c r="B34" s="30">
-        <f>IFERROR((B13+B14)/B9*100,"")</f>
+        <f>IFERROR((B13+B14)/B5*100,"")</f>
         <v/>
       </c>
       <c r="C34" s="30">
-        <f>IFERROR((C13+C14)/C9*100,"")</f>
+        <f>IFERROR((C13+C14)/C5*100,"")</f>
         <v/>
       </c>
       <c r="D34" s="30">
-        <f>IFERROR((D13+D14)/D9*100,"")</f>
+        <f>IFERROR((D13+D14)/D5*100,"")</f>
         <v/>
       </c>
       <c r="F34" s="29" t="n"/>
@@ -6157,19 +6177,19 @@
     <row r="35">
       <c r="A35" s="23" t="inlineStr">
         <is>
-          <t>Aktivernes omsætningshastighed (af bruttofortjeneste), gange</t>
+          <t>Aktivernes omsætningshastighed, gange</t>
         </is>
       </c>
       <c r="B35" s="30">
-        <f>IFERROR(B9/B21,"")</f>
+        <f>IFERROR(B5/B21,"")</f>
         <v/>
       </c>
       <c r="C35" s="30">
-        <f>IFERROR(C9/C21,"")</f>
+        <f>IFERROR(C5/C21,"")</f>
         <v/>
       </c>
       <c r="D35" s="30">
-        <f>IFERROR(D9/D21,"")</f>
+        <f>IFERROR(D5/D21,"")</f>
         <v/>
       </c>
       <c r="F35" s="29" t="n"/>
@@ -6255,19 +6275,19 @@
     <row r="41">
       <c r="A41" s="23" t="inlineStr">
         <is>
-          <t>Bruttofortjeneste</t>
+          <t>Nettoomsætning</t>
         </is>
       </c>
       <c r="B41" s="31">
-        <f>IFERROR(B9/$D9*100,"")</f>
+        <f>IFERROR(B5/$D5*100,"")</f>
         <v/>
       </c>
       <c r="C41" s="31">
-        <f>IFERROR(C9/$D9*100,"")</f>
+        <f>IFERROR(C5/$D5*100,"")</f>
         <v/>
       </c>
       <c r="D41" s="31">
-        <f>IFERROR(D9/$D9*100,"")</f>
+        <f>IFERROR(D5/$D5*100,"")</f>
         <v/>
       </c>
       <c r="F41" s="29" t="n"/>
@@ -6373,19 +6393,19 @@
     <row r="48">
       <c r="A48" s="23" t="inlineStr">
         <is>
-          <t>Bruttofortjeneste</t>
+          <t>Nettoomsætning</t>
         </is>
       </c>
       <c r="B48" s="31">
-        <f>IFERROR(B9*100/$D9,"")</f>
+        <f>IFERROR(B5*100/$D5,"")</f>
         <v/>
       </c>
       <c r="C48" s="31">
-        <f>IFERROR(C9*100/$D9,"")</f>
+        <f>IFERROR(C5*100/$D5,"")</f>
         <v/>
       </c>
       <c r="D48" s="31">
-        <f>IFERROR(D9*100/$D9,"")</f>
+        <f>IFERROR(D5*100/$D5,"")</f>
         <v/>
       </c>
       <c r="F48" s="29" t="n"/>
@@ -6722,7 +6742,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -7315,28 +7335,28 @@
       </c>
       <c r="B18" s="37" t="inlineStr">
         <is>
-          <t>ifrs-full:RevenueFromRenderingOfGamingServices</t>
+          <t>ifrs-full:TaxExpenseOtherThanIncomeTaxExpense</t>
         </is>
       </c>
       <c r="C18" s="37" t="inlineStr">
         <is>
-          <t>ifrs-full:RevenueFromRenderingOfGamingServices</t>
+          <t>ifrs-full:TaxExpenseOtherThanIncomeTaxExpense</t>
         </is>
       </c>
       <c r="D18" s="38" t="n">
-        <v>1819679</v>
+        <v>513868</v>
       </c>
       <c r="E18" s="38" t="n">
-        <v>1661743</v>
+        <v>471559</v>
       </c>
       <c r="F18" s="38" t="n">
-        <v>1613015</v>
+        <v>456874</v>
       </c>
       <c r="G18" s="38" t="n">
-        <v>1631692</v>
+        <v>466806</v>
       </c>
       <c r="H18" s="38" t="n">
-        <v>1584199</v>
+        <v>450699</v>
       </c>
       <c r="I18" s="39" t="inlineStr">
         <is>
@@ -7352,63 +7372,26 @@
       </c>
       <c r="B19" s="34" t="inlineStr">
         <is>
-          <t>ifrs-full:TaxExpenseOtherThanIncomeTaxExpense</t>
+          <t>ifrs-full:TradeAndOtherCurrentReceivablesDueFromRelatedParties</t>
         </is>
       </c>
       <c r="C19" s="34" t="inlineStr">
         <is>
-          <t>ifrs-full:TaxExpenseOtherThanIncomeTaxExpense</t>
+          <t>ifrs-full:TradeAndOtherCurrentReceivablesDueFromRelatedParties</t>
         </is>
       </c>
       <c r="D19" s="35" t="n">
-        <v>513868</v>
+        <v>122495</v>
       </c>
       <c r="E19" s="35" t="n">
-        <v>471559</v>
-      </c>
-      <c r="F19" s="35" t="n">
-        <v>456874</v>
-      </c>
-      <c r="G19" s="35" t="n">
-        <v>466806</v>
-      </c>
+        <v>160543</v>
+      </c>
+      <c r="F19" s="35" t="n"/>
+      <c r="G19" s="35" t="n"/>
       <c r="H19" s="35" t="n">
-        <v>450699</v>
+        <v>282980</v>
       </c>
       <c r="I19" s="36" t="inlineStr">
-        <is>
-          <t>Ingen forklaring tilgængelig.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="37" t="inlineStr">
-        <is>
-          <t>Øvrige (ukendt)</t>
-        </is>
-      </c>
-      <c r="B20" s="37" t="inlineStr">
-        <is>
-          <t>ifrs-full:TradeAndOtherCurrentReceivablesDueFromRelatedParties</t>
-        </is>
-      </c>
-      <c r="C20" s="37" t="inlineStr">
-        <is>
-          <t>ifrs-full:TradeAndOtherCurrentReceivablesDueFromRelatedParties</t>
-        </is>
-      </c>
-      <c r="D20" s="38" t="n">
-        <v>122495</v>
-      </c>
-      <c r="E20" s="38" t="n">
-        <v>160543</v>
-      </c>
-      <c r="F20" s="38" t="n"/>
-      <c r="G20" s="38" t="n"/>
-      <c r="H20" s="38" t="n">
-        <v>282980</v>
-      </c>
-      <c r="I20" s="39" t="inlineStr">
         <is>
           <t>Ingen forklaring tilgængelig.</t>
         </is>

</xml_diff>